<commit_message>
acabando nos onepages e emails
</commit_message>
<xml_diff>
--- a/prospecção/abordagem/alvos_prioritarios.xlsx
+++ b/prospecção/abordagem/alvos_prioritarios.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prioritários" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritários'!$A$1:$U$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prioritários'!$A$1:$U$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U51"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -572,30 +572,30 @@
       <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EUROINVEST S.A. CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS</t>
+          <t>EBADIVAL - E. BAGGIO DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Rio De Janeiro</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2117963.09</v>
+        <v>758266.8</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1989</t>
+          <t>1978</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -612,15 +612,19 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>EUROINVEST@GRUPOEUROINVEST.COM.BR</t>
+          <t>EBADIVAL@EBADIVAL.COM.BR</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>21 22248653</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+          <t>41 33732020</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>WWW.EBADIVAL.COM.BR</t>
+        </is>
+      </c>
       <c r="O2" s="3" t="inlineStr"/>
       <c r="P2" s="3" t="inlineStr"/>
       <c r="Q2" s="3" t="inlineStr"/>
@@ -633,30 +637,30 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LEVYCAM - CORRETORA DE CAMBIO E VALORES LTDA.</t>
+          <t>FIDUCIAL DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Belo Horizonte</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>9827342.32</v>
+        <v>969463.78</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1982</t>
+          <t>2008</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -673,17 +677,17 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>LEVYCAM@LEVYCAM.COM.BR</t>
+          <t>RODRIGO@FIDUCIAL.COM.BR</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>11 28139600</t>
+          <t>31 21057600</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>WWW.LEVYCAM.COM.BR</t>
+          <t>WWW.FIDUCIAL.COM.BR</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr"/>
@@ -698,7 +702,7 @@
       <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ACTIVTRADES CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
+          <t>EUROINVEST S.A. CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -708,20 +712,20 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Florianópolis</t>
+          <t>Rio De Janeiro</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>12333491.41</v>
+        <v>2117963.09</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>1989</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -738,19 +742,15 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>AOLIVEIRA@ACTIVTRADES.COM</t>
+          <t>EUROINVEST@GRUPOEUROINVEST.COM.BR</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>48 31126700</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>WWW.ACTIVTRADES.COM.BR</t>
-        </is>
-      </c>
+          <t>21 22248653</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
       <c r="O4" s="3" t="inlineStr"/>
       <c r="P4" s="3" t="inlineStr"/>
       <c r="Q4" s="3" t="inlineStr"/>
@@ -763,30 +763,30 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AMARIL FRANKLIN CORRETORA DE TÍTULOS E VALORES LTDA</t>
+          <t>DEBONI DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS LTDA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>16432954.97</v>
+        <v>2250685.08</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1976</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -803,17 +803,17 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>INVESTIMENTOS@AMARILFRANKLIN.COM.BR</t>
+          <t>DEBONI@HOTMAIL.COM</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>31 32358100</t>
+          <t>41 999838800</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>WWW.AMARILFRANKLIN.COM.BR</t>
+          <t>WWW.DEBONICAMBIO.COM.BR</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr"/>
@@ -828,30 +828,30 @@
       <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BPY CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
+          <t>PACIFIC INVEST DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS LTDA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Joaçaba</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>20063943.7</v>
+        <v>2534246.63</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>1993</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -868,17 +868,17 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>CONTATO@BPY.GLOBAL</t>
+          <t>ADMINISTRATIVO@PACIFICINVEST.COM.BR</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>11 29702933</t>
+          <t>49 35222580</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>WWW.IBCORRETORA.COM.BR</t>
+          <t>HTTP://WWW.PACIFICINVEST.COM.BR</t>
         </is>
       </c>
       <c r="O6" s="3" t="inlineStr"/>
@@ -893,12 +893,12 @@
       <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SENSO CORRETORA DE CAMBIO E VALORES MOBILIARIOS S.A</t>
+          <t>MOMENTO DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS LTDA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>21983750.53</v>
+        <v>3119089.65</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>1994</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -933,19 +933,15 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>SENSO@SENSOCORRETORA.COM.BR</t>
+          <t>LAGRA@SAOCLEMENTESA.COM.BR</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>21 25055000</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>WWW.SENSOCORRETORA.COM.BR</t>
-        </is>
-      </c>
+          <t>21 32666666</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
       <c r="O7" s="3" t="inlineStr"/>
       <c r="P7" s="3" t="inlineStr"/>
       <c r="Q7" s="3" t="inlineStr"/>
@@ -958,30 +954,30 @@
       <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SOCIAL BANK BANCO MÚLTIPLO S/A</t>
+          <t>GLOBAL INVESTMENT SERVICES DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Salvador</t>
+          <t>São Paulo</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>22087181.62</v>
+        <v>3465875.82</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1943</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -998,19 +994,15 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>COMPLIANCE@SOCIALBANK.COM.BR</t>
+          <t>COMPLIANCE@MOGNODTVM.COM</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>71 21041000</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>HTTPS://WWW.SOCIALBANK.COM.BR/</t>
-        </is>
-      </c>
+          <t>800 1608</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" s="3" t="inlineStr"/>
       <c r="P8" s="3" t="inlineStr"/>
       <c r="Q8" s="3" t="inlineStr"/>
@@ -1023,12 +1015,12 @@
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BANCO PORTO REAL DE INVESTIMENTOS S.A</t>
+          <t>GDC PARTNERS SERVIÇOS FIDUCIÁRIOS DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Banco de Investimento</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1038,15 +1030,15 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Porto Real</t>
+          <t>Rio De Janeiro</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>30736757.87</v>
+        <v>3620789.76</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1992</t>
+          <t>2009</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1063,12 +1055,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>FINANBPR@BPR.COM.BR</t>
+          <t>GDC@GDCDTVM.COM.BR</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>24 20320002</t>
+          <t>21 24904305</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
@@ -1084,12 +1076,12 @@
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BANCO CEDULA S.A.</t>
+          <t>BCP SECURITIES DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1103,11 +1095,11 @@
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>32908577.68</v>
+        <v>4469865.46</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1965</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1124,17 +1116,17 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>BANCOCEDULA@BANCOCEDULA.COM.BR</t>
+          <t>BORLANDINI@BCPSECURITIES.COM</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>21 22215512</t>
+          <t>21 22274160</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>WWW.BANCOCEDULA.COM.BR</t>
+          <t>HTTPS://BCPDTVM.COM.BR/</t>
         </is>
       </c>
       <c r="O10" s="3" t="inlineStr"/>
@@ -1149,12 +1141,12 @@
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SIMPAUL CORRETORA DE CAMBIO E VALORES MOBILIARIOS  S.A.</t>
+          <t>CAROL DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS LTDA.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1168,16 +1160,16 @@
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>45519071.58</v>
+        <v>4633259.43</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>1993</t>
+          <t>1968</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1189,19 +1181,15 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>CONTROLESINTERNOS@SIMPAUL.COM.BR</t>
+          <t>KLEBER@CAROLDTVM.COM.BR</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>51 33279888</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>WWW.SIMPAUL.COM.BR</t>
-        </is>
-      </c>
+          <t>11 22278899</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
       <c r="O11" s="3" t="inlineStr"/>
       <c r="P11" s="3" t="inlineStr"/>
       <c r="Q11" s="3" t="inlineStr"/>
@@ -1214,12 +1202,12 @@
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BANCO INDUSCRED DE INVESTIMENTO S.A.</t>
+          <t>LEV DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Banco de Investimento</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1233,16 +1221,16 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>51108343.25</v>
+        <v>7395806.02</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>1941</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>já custodia</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1254,17 +1242,17 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>CONTATO@BANCOINDUSCRED.COM.BR</t>
+          <t>MARCELO.CERIZE@LEV.COM.VC</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>11 31912000</t>
+          <t>11 40406610</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>WWW.BANCOINDUSCRED.COM.BR</t>
+          <t>HTTPS://WWW.LEV.COM.VC/</t>
         </is>
       </c>
       <c r="O12" s="3" t="inlineStr"/>
@@ -1279,30 +1267,30 @@
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
-          <t>H H PICCHIONI S/A CORRETORA DE CAMBIO E VALORES MOBILIARIOS</t>
+          <t>PENTAGONO S/A DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Belo Horizonte</t>
+          <t>Rio De Janeiro</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>58710307.07</v>
+        <v>7735221.03</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1967</t>
+          <t>1968</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1319,17 +1307,17 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>PICCHIONI@PICCHIONI.COM.BR</t>
+          <t>DIRETORIA@PENTAGONOTRUSTEE.COM.BR</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>31 32387126</t>
+          <t>21 33854565</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>WWW.PICCHIONI.COM.BR</t>
+          <t>WWW.PENTAGONOTRUSTEE.COM.BR</t>
         </is>
       </c>
       <c r="O13" s="3" t="inlineStr"/>
@@ -1344,30 +1332,30 @@
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BANCO RNX S.A.</t>
+          <t>UNICRED DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS LTDA</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>118736076.42</v>
+        <v>8369773.98</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>1987</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1384,17 +1372,13 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>BANCORNX@BANCORNX.COM.BR</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>41 30745900</t>
-        </is>
-      </c>
+          <t>DTVM@UNICRED.COM.BR</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>WWW.BANCORNX.COM.BR</t>
+          <t>WWW.UNICRED.COM.BR</t>
         </is>
       </c>
       <c r="O14" s="3" t="inlineStr"/>
@@ -1409,7 +1393,7 @@
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CM CAPITAL MARKETS CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS LTDA</t>
+          <t>LEVYCAM - CORRETORA DE CAMBIO E VALORES LTDA.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1428,16 +1412,16 @@
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>131100402.32</v>
+        <v>9827342.32</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1998</t>
+          <t>1982</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -1449,17 +1433,17 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>GOVERNANCA@CMCAPITAL.COM.BR</t>
+          <t>LEVYCAM@LEVYCAM.COM.BR</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>11 38421122</t>
+          <t>11 28139600</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>WWW.CMCAPITAL.COM.BR</t>
+          <t>WWW.LEVYCAM.COM.BR</t>
         </is>
       </c>
       <c r="O15" s="3" t="inlineStr"/>
@@ -1474,12 +1458,12 @@
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
-          <t>EQI INVESTIMENTOS CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
+          <t>AZIMUT BRASIL DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1493,16 +1477,16 @@
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>133653144.25</v>
+        <v>10909296.91</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2013</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>já custodia</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -1514,15 +1498,19 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>NOTIFICACOES.REGULATORIO@EQI.COM.BR</t>
+          <t>COMPLIANCE@AZIMUTBRASIL.COM</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>47 984490035</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr"/>
+          <t>11 35527656</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>HTTP://WWW.AZIMUTBRASIL.COM.BR/AZWEALTH/</t>
+        </is>
+      </c>
       <c r="O16" s="3" t="inlineStr"/>
       <c r="P16" s="3" t="inlineStr"/>
       <c r="Q16" s="3" t="inlineStr"/>
@@ -1535,12 +1523,12 @@
       <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MONTE BRAVO CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
+          <t>WEALTH HIGH GOVERNANCE DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1554,7 +1542,7 @@
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>201587382.81</v>
+        <v>11250528.43</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1566,11 +1554,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
@@ -1579,17 +1563,17 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>CAIO.RIZK@MONTEBRAVO.COM.BR</t>
+          <t>ERIC.CARDOZO@WHG.COM.BR</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>11 30180960</t>
+          <t>11 35092322</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>WWW.MONTEBRAVO.COM.BR</t>
+          <t>HTTPS://WHG.COM.BR/</t>
         </is>
       </c>
       <c r="O17" s="3" t="inlineStr"/>
@@ -1604,30 +1588,30 @@
       <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AVENUE SECURITIES BANCO DE INVESTIMENTO S.A.</t>
+          <t>NIKOS DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Banco de Investimento</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>São Paulo</t>
+          <t>Rio De Janeiro</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>237784221.46</v>
+        <v>11603299.77</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>1989</t>
+          <t>1981</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1644,19 +1628,15 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>REGULATORIO@AVENUE.US</t>
+          <t>JURIDICO@NIKOS.COM.BR</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>11 23855535</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>HTTPS://DTVM.AVENUE.US/</t>
-        </is>
-      </c>
+          <t>21 995069870</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
       <c r="O18" s="3" t="inlineStr"/>
       <c r="P18" s="3" t="inlineStr"/>
       <c r="Q18" s="3" t="inlineStr"/>
@@ -1669,26 +1649,32 @@
       <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BANCO NACIONAL S.A.</t>
+          <t>ACTIVTRADES CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Rio De Janeiro</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+          <t>Florianópolis</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>12333491.41</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>—</t>
@@ -1703,15 +1689,19 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>bnsa@bnsa.com.br</t>
+          <t>AOLIVEIRA@ACTIVTRADES.COM</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>21 39832321</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr"/>
+          <t>48 31126700</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>WWW.ACTIVTRADES.COM.BR</t>
+        </is>
+      </c>
       <c r="O19" s="3" t="inlineStr"/>
       <c r="P19" s="3" t="inlineStr"/>
       <c r="Q19" s="3" t="inlineStr"/>
@@ -1724,12 +1714,12 @@
       <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BANCO BRADESCARD S.A.</t>
+          <t>H.COMMCOR DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1739,11 +1729,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Osasco</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>16010658.7</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>—</t>
@@ -1758,17 +1754,17 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>5404.REGULATORIO@BRADESCO.COM.BR</t>
+          <t>DIRETORIA@COMMCOR.COM.BR</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>11 48313499</t>
+          <t>11 21272727</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>HTTPS://WWW.BRADESCARD.COM.BR</t>
+          <t>WWW.COMMCOR.COM.BR</t>
         </is>
       </c>
       <c r="O20" s="3" t="inlineStr"/>
@@ -1783,12 +1779,12 @@
       <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
-          <t>KIRTON BANK S.A. - BANCO MÚLTIPLO</t>
+          <t>TRADERS DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1798,14 +1794,20 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Osasco</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>16171692.17</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1968</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>já custodia</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -1817,15 +1819,19 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>OUVIDORIA.BRA@BRADESCO.COM.BR</t>
+          <t>INSTITUCIONAL@TRADERS.COM.BR</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>41 37776161</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr"/>
+          <t>11 23951100</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>WWW.TRADERS.COM.BR</t>
+        </is>
+      </c>
       <c r="O21" s="3" t="inlineStr"/>
       <c r="P21" s="3" t="inlineStr"/>
       <c r="Q21" s="3" t="inlineStr"/>
@@ -1838,26 +1844,32 @@
       <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BANCO LOSANGO S.A. - BANCO MÚLTIPLO</t>
+          <t>AMARIL FRANKLIN CORRETORA DE TÍTULOS E VALORES LTDA</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Rio De Janeiro</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>16432954.97</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>—</t>
@@ -1872,17 +1884,17 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>GUILHERME.PIEDADE@BRADESCO.COM.BR</t>
+          <t>INVESTIMENTOS@AMARILFRANKLIN.COM.BR</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>11 55037500</t>
+          <t>31 32358100</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>WWW2.LOSANGO.COM.BR</t>
+          <t>WWW.AMARILFRANKLIN.COM.BR</t>
         </is>
       </c>
       <c r="O22" s="3" t="inlineStr"/>
@@ -1897,26 +1909,32 @@
       <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BANCO BANDEPE S.A.</t>
+          <t>COLUNA S/A DISTRIBUIDORA DE TITULOS E VALORES MOBILIÁRIOS</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+          <t>Rio De Janeiro</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>18292027.37</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>—</t>
@@ -1931,17 +1949,17 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>CORGREGULADORES@SANTANDER.COM.BR</t>
+          <t>COMPLIANCE@COLUNADTVM.COM.BR</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>11 35535533</t>
+          <t>21 25050300</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>HTTPS://WWW.SANTANDER.COM.BR</t>
+          <t>WWW.COLUNADTVM.COM.BR</t>
         </is>
       </c>
       <c r="O23" s="3" t="inlineStr"/>
@@ -1956,26 +1974,32 @@
       <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
-          <t>OMNI BANCO S.A.</t>
+          <t>OPPORTUNITY DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+          <t>Rio De Janeiro</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>19271502.67</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>—</t>
@@ -1990,19 +2014,15 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>OMNI.BANCO@OMNI.COM.BR</t>
+          <t>GAR.DTVM@OPPORTUNITY.COM.BR</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>11 33653522</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>HTTPS://REBRAND.LY/WHATSAPPOUVIDORIAOMNI</t>
-        </is>
-      </c>
+          <t>21 38043800</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
       <c r="O24" s="3" t="inlineStr"/>
       <c r="P24" s="3" t="inlineStr"/>
       <c r="Q24" s="3" t="inlineStr"/>
@@ -2015,12 +2035,12 @@
       <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BANCO CAIXA GERAL - BRASIL S.A.</t>
+          <t>BPY CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2033,15 +2053,17 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="n">
+        <v>20063943.7</v>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>1938</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -2053,17 +2075,17 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>BCGBRASIL@BCGBRASIL.COM.BR</t>
+          <t>CONTATO@BPY.GLOBAL</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>11 35099300</t>
+          <t>11 29702933</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>WWW.BCGBRASIL.COM.BR</t>
+          <t>WWW.IBCORRETORA.COM.BR</t>
         </is>
       </c>
       <c r="O25" s="3" t="inlineStr"/>
@@ -2078,33 +2100,35 @@
       <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BANCO SOFISA S.A.</t>
+          <t>SENSO CORRETORA DE CAMBIO E VALORES MOBILIARIOS S.A</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>Rio De Janeiro</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>21983750.53</v>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>1961</t>
+          <t>1968</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -2116,17 +2140,17 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>INSTITUCIONALSOFISABCB@SOFISA.COM.BR</t>
+          <t>SENSO@SENSOCORRETORA.COM.BR</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>11 31765500</t>
+          <t>21 25055000</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>WWW.SOFISA.COM.BR</t>
+          <t>WWW.SENSOCORRETORA.COM.BR</t>
         </is>
       </c>
       <c r="O26" s="3" t="inlineStr"/>
@@ -2141,26 +2165,32 @@
       <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BANCO INVESTCRED UNIBANCO S.A.</t>
+          <t>SOCIAL BANK BANCO MÚLTIPLO S/A</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Banco Comercial</t>
+          <t>Banco Múltiplo</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>22087181.62</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>1943</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>—</t>
@@ -2175,17 +2205,17 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>RELACIONAMENTO.BACEN@ITAU-UNIBANCO.COM.BR</t>
+          <t>COMPLIANCE@SOCIALBANK.COM.BR</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>11 50199968</t>
+          <t>71 21041000</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>WWW.ITAU.COM.BR</t>
+          <t>HTTPS://WWW.SOCIALBANK.COM.BR/</t>
         </is>
       </c>
       <c r="O27" s="3" t="inlineStr"/>
@@ -2200,26 +2230,32 @@
       <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BANCO BESA S.A.</t>
+          <t>BANCO PORTO REAL DE INVESTIMENTOS S.A</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Banco de Investimento</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+          <t>Porto Real</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>30736757.87</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>1992</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>—</t>
@@ -2234,12 +2270,12 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>ATENDIMENTO@BANCOBESA.COM.BR</t>
+          <t>FINANBPR@BPR.COM.BR</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>11 33264824</t>
+          <t>24 20320002</t>
         </is>
       </c>
       <c r="N28" t="inlineStr"/>
@@ -2255,7 +2291,7 @@
       <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BANCO SANY BRASIL S.A.</t>
+          <t>BANCO CEDULA S.A.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2265,16 +2301,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+          <t>Rio De Janeiro</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>32908577.68</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1965</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>—</t>
@@ -2289,11 +2331,19 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>ANDRADEL@SANYGROUP.COM</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
+          <t>BANCOCEDULA@BANCOCEDULA.COM.BR</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>21 22215512</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>WWW.BANCOCEDULA.COM.BR</t>
+        </is>
+      </c>
       <c r="O29" s="3" t="inlineStr"/>
       <c r="P29" s="3" t="inlineStr"/>
       <c r="Q29" s="3" t="inlineStr"/>
@@ -2306,12 +2356,12 @@
       <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BANCO ABN AMRO CLEARING S.A.</t>
+          <t>UNIDA DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2321,18 +2371,20 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr"/>
+          <t>Barueri</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>33406013.31</v>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>1968</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -2344,19 +2396,15 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>COMPLIANCE.BR@ABNAMROCLEARING.COM</t>
+          <t>COMPLIANCE-CI@UNIDADTVM.COM.BR</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>11 30737400</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>HTTPS://WWW.ABNAMRO.COM/BR/PT/HOME</t>
-        </is>
-      </c>
+          <t>11 35065500</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr"/>
       <c r="O30" s="3" t="inlineStr"/>
       <c r="P30" s="3" t="inlineStr"/>
       <c r="Q30" s="3" t="inlineStr"/>
@@ -2369,12 +2417,12 @@
       <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BANCO VR S.A.</t>
+          <t>F.D'GOLD - DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2387,10 +2435,12 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="n">
+        <v>44200062.71</v>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>1968</t>
+          <t>2007</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2407,19 +2457,15 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>COMPLIANCE@BANCOVR.COM.BR</t>
+          <t>JOAO.OLIVEIRA@DGOLD.COM.BR</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>11 41347500</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>WWW.BANCOVR.COM.BR</t>
-        </is>
-      </c>
+          <t>11 35495070</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
       <c r="O31" s="3" t="inlineStr"/>
       <c r="P31" s="3" t="inlineStr"/>
       <c r="Q31" s="3" t="inlineStr"/>
@@ -2432,12 +2478,12 @@
       <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BANCO TRATON BRASIL S.A.</t>
+          <t>SIMPAUL CORRETORA DE CAMBIO E VALORES MOBILIARIOS  S.A.</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2450,11 +2496,17 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
+      <c r="F32" s="2" t="n">
+        <v>45519071.58</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>já custodia</t>
         </is>
       </c>
       <c r="I32" t="inlineStr"/>
@@ -2466,15 +2518,19 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>EDUARDO.PORTAS@TRATONFS.COM</t>
+          <t>CONTROLESINTERNOS@SIMPAUL.COM.BR</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>11 983543751</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr"/>
+          <t>51 33279888</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>WWW.SIMPAUL.COM.BR</t>
+        </is>
+      </c>
       <c r="O32" s="3" t="inlineStr"/>
       <c r="P32" s="3" t="inlineStr"/>
       <c r="Q32" s="3" t="inlineStr"/>
@@ -2487,12 +2543,12 @@
       <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BANCOSEGURO S.A.</t>
+          <t>OM DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2505,11 +2561,17 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+      <c r="F33" s="2" t="n">
+        <v>47163195.73</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
@@ -2521,17 +2583,17 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>REGULATORIO@UOLINC.COM</t>
+          <t>COMPLIANCE@OUROMINAS.COM</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>11 40031775</t>
+          <t>11 32180991</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>HTTPS://PAGSEGURO.VC/OUVIDORIA</t>
+          <t>HTTPS://OUROMINAS.COM/OM</t>
         </is>
       </c>
       <c r="O33" s="3" t="inlineStr"/>
@@ -2546,12 +2608,12 @@
       <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BANCO DA CHINA BRASIL S.A.</t>
+          <t>HEDGEPOINT GLOBAL MARKETS DISTRIBUIDORA DE TITULOS E VALORES MOBILIÁRIOS LTDA.</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2561,11 +2623,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
+          <t>Campinas</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>49216586</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
           <t>—</t>
@@ -2580,19 +2648,15 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>CONTATOBC@BOC-BRAZIL.COM</t>
+          <t>EDUARDO.ROEDEL@HEDGEPOINTGLOBAL.COM</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>11 35083200</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>HTTPS://WWW.BANKOFCHINA.COM/BR/PT/</t>
-        </is>
-      </c>
+          <t>11 9961300400</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
       <c r="O34" s="3" t="inlineStr"/>
       <c r="P34" s="3" t="inlineStr"/>
       <c r="Q34" s="3" t="inlineStr"/>
@@ -2605,28 +2669,30 @@
       <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PARANÁ BANCO S.A.</t>
+          <t>BANCO INDUSCRED DE INVESTIMENTO S.A.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Banco de Investimento</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>51108343.25</v>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1941</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2643,17 +2709,17 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>PRESIDENCIA@PARANABANCO.COM.BR</t>
+          <t>CONTATO@BANCOINDUSCRED.COM.BR</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>41 33519899</t>
+          <t>11 31912000</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>WWW.PARANABANCO.COM.BR</t>
+          <t>WWW.BANCOINDUSCRED.COM.BR</t>
         </is>
       </c>
       <c r="O35" s="3" t="inlineStr"/>
@@ -2668,28 +2734,30 @@
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BANCO BARI DE INVESTIMENTOS E FINANCIAMENTOS S.A.</t>
+          <t>RB INVESTIMENTOS DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS LIMITADA</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>57840463.52</v>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>1983</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -2706,17 +2774,17 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>COMPLIANCE@BANCOBARI.COM.BR</t>
+          <t>COMPLIANCE@RBINVESTIMENTOS.COM</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>41 40072628</t>
+          <t>11 31272700</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>WWW.BANCOBARI.COM.BR</t>
+          <t>WWW.RBINVESTIMENTOS.COM</t>
         </is>
       </c>
       <c r="O36" s="3" t="inlineStr"/>
@@ -2731,26 +2799,32 @@
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
-          <t>BANCO SISTEMA S.A.</t>
+          <t>H H PICCHIONI S/A CORRETORA DE CAMBIO E VALORES MOBILIARIOS</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Banco Múltiplo</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Curitiba</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>58710307.07</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>—</t>
@@ -2765,17 +2839,17 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>OUVIDORIA@BANCOSISTEMA.COM.BR</t>
+          <t>PICCHIONI@PICCHIONI.COM.BR</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>41 35253812</t>
+          <t>31 32387126</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>WWW.BTGPACTUAL.COM</t>
+          <t>WWW.PICCHIONI.COM.BR</t>
         </is>
       </c>
       <c r="O37" s="3" t="inlineStr"/>
@@ -2790,12 +2864,12 @@
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CODEPE CORRETORA DE VALORES E CÂMBIO S.A.</t>
+          <t>GALAPAGOS CAPITAL DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2805,13 +2879,15 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Barueri</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>115632423.58</v>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2828,19 +2904,15 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>CODEPE@CODEPE.COM.BR</t>
+          <t>COMPLIANCE@GALAPAGOSCAPITAL.COM</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>81 21377979</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>WWW.CODEPE.COM.BR</t>
-        </is>
-      </c>
+          <t>11 37772088</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr"/>
       <c r="O38" s="3" t="inlineStr"/>
       <c r="P38" s="3" t="inlineStr"/>
       <c r="Q38" s="3" t="inlineStr"/>
@@ -2853,33 +2925,35 @@
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TULLETT PREBON BRASIL CORRETORA DE VALORES E CÂMBIO LTDA</t>
+          <t>BANCO RNX S.A.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Banco Múltiplo</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
+          <t>Curitiba</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>118736076.42</v>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2008</t>
+          <t>1987</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I39" t="inlineStr"/>
@@ -2891,17 +2965,17 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>PEDRO.FERNANDES@BR.ICAP.COM</t>
+          <t>BANCORNX@BANCORNX.COM.BR</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>11 21114800</t>
+          <t>41 30745900</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>TULLETTPREBON.COM.BR</t>
+          <t>WWW.BANCORNX.COM.BR</t>
         </is>
       </c>
       <c r="O39" s="3" t="inlineStr"/>
@@ -2916,7 +2990,7 @@
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MERRILL LYNCH S.A. CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS</t>
+          <t>CM CAPITAL MARKETS CORRETORA DE CÂMBIO, TÍTULOS E VALORES MOBILIÁRIOS LTDA</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2934,8 +3008,14 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
+      <c r="F40" s="2" t="n">
+        <v>131100402.32</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>já custodia</t>
@@ -2950,17 +3030,17 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>DG.BRAZIL_LOB_COR@BANKOFAMERICA.COM</t>
+          <t>GOVERNANCA@CMCAPITAL.COM.BR</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>11 21884000</t>
+          <t>11 38421122</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>HTTPS://WWW.BOFABRASIL.COM.BR/</t>
+          <t>WWW.CMCAPITAL.COM.BR</t>
         </is>
       </c>
       <c r="O40" s="3" t="inlineStr"/>
@@ -2975,26 +3055,32 @@
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BANCO NACIONAL DE INVESTIMENTOS S.A.</t>
+          <t>EQI INVESTIMENTOS CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Banco de Investimento</t>
+          <t>Sociedade Corretora de TVM</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Rio De Janeiro</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n">
+        <v>133653144.25</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>—</t>
@@ -3009,12 +3095,12 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>bnsa@bnsa.com.br</t>
+          <t>NOTIFICACOES.REGULATORIO@EQI.COM.BR</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>21 39832321</t>
+          <t>47 984490035</t>
         </is>
       </c>
       <c r="N41" t="inlineStr"/>
@@ -3030,7 +3116,7 @@
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ICAP DO BRASIL CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
+          <t>MONTE BRAVO CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -3040,22 +3126,32 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Rio De Janeiro</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>201587382.81</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>já custodia</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr">
         <is>
@@ -3064,15 +3160,19 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>PEDRO.FERNANDES@BR.ICAP.COM</t>
+          <t>CAIO.RIZK@MONTEBRAVO.COM.BR</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>21 39564200</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr"/>
+          <t>11 30180960</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>WWW.MONTEBRAVO.COM.BR</t>
+        </is>
+      </c>
       <c r="O42" s="3" t="inlineStr"/>
       <c r="P42" s="3" t="inlineStr"/>
       <c r="Q42" s="3" t="inlineStr"/>
@@ -3085,7 +3185,7 @@
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BB-BANCO DE INVESTIMENTO S/A</t>
+          <t>AVENUE SECURITIES BANCO DE INVESTIMENTO S.A.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3103,11 +3203,17 @@
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
+      <c r="F43" s="2" t="n">
+        <v>237784221.46</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>já custodia</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
@@ -3119,17 +3225,17 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>BBBI.GOV@BB.COM.BR</t>
+          <t>REGULATORIO@AVENUE.US</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>11 42987042</t>
+          <t>11 23855535</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>WWW.BB.COM.BR</t>
+          <t>HTTPS://DTVM.AVENUE.US/</t>
         </is>
       </c>
       <c r="O43" s="3" t="inlineStr"/>
@@ -3144,26 +3250,32 @@
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ÁGORA CORRETORA DE TITULOS E VALORES MOBILIARIOS S.A.</t>
+          <t>BGC LIQUIDEZ DISTRIBUIDORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+          <t>Rio De Janeiro</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>274077948.04</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>1968</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>já custodia</t>
@@ -3178,17 +3290,17 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>CARLOSEDUARDO.VIANNA@AGORAINVESTIMENTOS.COM.BR</t>
+          <t>LIQUIDEZ-BACEN@BGCG.COM</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>21 25290800</t>
+          <t>21 30433000</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>WWW.AGORAINVEST.COM.BR</t>
+          <t>WWW.BGCLIQUIDEZ.COM</t>
         </is>
       </c>
       <c r="O44" s="3" t="inlineStr"/>
@@ -3203,26 +3315,32 @@
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PAGINVEST CORRETORA DE TITULOS E VALORES MOBILIARIOS LTDA.</t>
+          <t>VIC-DISTRIBUIDORA DE TITULOS E VALORES MOBILIARIOS S/A</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Sociedade Corretora de TVM</t>
+          <t>Sociedade Distribuidora de TVM</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+          <t>Rio De Janeiro</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>300724345.83</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>1977</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>já custodia</t>
@@ -3237,19 +3355,15 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>REGULATORIO@UOLINC.COM</t>
+          <t>VICADLER@UOL.COM.BR</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>11 30389285</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>HTTPS://PAGSEGURO.VC/OUVIDORIA</t>
-        </is>
-      </c>
+          <t>21 39709250</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
       <c r="O45" s="3" t="inlineStr"/>
       <c r="P45" s="3" t="inlineStr"/>
       <c r="Q45" s="3" t="inlineStr"/>
@@ -3258,362 +3372,8 @@
       <c r="T45" s="3" t="inlineStr"/>
       <c r="U45" s="3" t="inlineStr"/>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>GURU CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Sociedade Corretora de TVM</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>Banco/CTVM</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>FELIPE@GURU.COM.VC</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>11 98144455</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>HTTPS://WWW.GURUCTVM.COM.BR/</t>
-        </is>
-      </c>
-      <c r="O46" s="3" t="inlineStr"/>
-      <c r="P46" s="3" t="inlineStr"/>
-      <c r="Q46" s="3" t="inlineStr"/>
-      <c r="R46" s="3" t="inlineStr"/>
-      <c r="S46" s="3" t="inlineStr"/>
-      <c r="T46" s="3" t="inlineStr"/>
-      <c r="U46" s="3" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>IDEAL CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Sociedade Corretora de TVM</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>já gere fundos + já custodia</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>Banco/CTVM</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>CONTATO@IDEALCTVM.COM.BR</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>11 30143545</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>WWW.IDEALCTVM.COM.BR</t>
-        </is>
-      </c>
-      <c r="O47" s="3" t="inlineStr"/>
-      <c r="P47" s="3" t="inlineStr"/>
-      <c r="Q47" s="3" t="inlineStr"/>
-      <c r="R47" s="3" t="inlineStr"/>
-      <c r="S47" s="3" t="inlineStr"/>
-      <c r="T47" s="3" t="inlineStr"/>
-      <c r="U47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>NEON CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS S.A.</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Sociedade Corretora de TVM</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>já custodia</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>Banco/CTVM</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>MARIANA.UVO@NEON.COM.BR</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>800 8820652</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>HTTPS://NEON.COM.BR/</t>
-        </is>
-      </c>
-      <c r="O48" s="3" t="inlineStr"/>
-      <c r="P48" s="3" t="inlineStr"/>
-      <c r="Q48" s="3" t="inlineStr"/>
-      <c r="R48" s="3" t="inlineStr"/>
-      <c r="S48" s="3" t="inlineStr"/>
-      <c r="T48" s="3" t="inlineStr"/>
-      <c r="U48" s="3" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>ABN AMRO CLEARING CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS LTDA.</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Sociedade Corretora de TVM</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>Banco/CTVM</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>COMPLIANCE.BR@ABNAMROCLEARING.COM</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>11 37037437</t>
-        </is>
-      </c>
-      <c r="N49" t="inlineStr">
-        <is>
-          <t>HTTPS://WWW.ABNAMRO.COM/BR/PT/HOME</t>
-        </is>
-      </c>
-      <c r="O49" s="3" t="inlineStr"/>
-      <c r="P49" s="3" t="inlineStr"/>
-      <c r="Q49" s="3" t="inlineStr"/>
-      <c r="R49" s="3" t="inlineStr"/>
-      <c r="S49" s="3" t="inlineStr"/>
-      <c r="T49" s="3" t="inlineStr"/>
-      <c r="U49" s="3" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>NU INVESTIMENTOS S.A. - CORRETORA DE TÍTULOS E VALORES MOBILIÁRIOS</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Sociedade Corretora de TVM</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>já custodia</t>
-        </is>
-      </c>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>Banco/CTVM</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>CHAPTER-LEGAL@NUBANK.COM.BR</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>11 38414510</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>HTTPS://WWW.NUINVEST.COM.BR/</t>
-        </is>
-      </c>
-      <c r="O50" s="3" t="inlineStr"/>
-      <c r="P50" s="3" t="inlineStr"/>
-      <c r="Q50" s="3" t="inlineStr"/>
-      <c r="R50" s="3" t="inlineStr"/>
-      <c r="S50" s="3" t="inlineStr"/>
-      <c r="T50" s="3" t="inlineStr"/>
-      <c r="U50" s="3" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>CGD INVESTIMENTOS CORRETORA DE VALORES E CÂMBIO S.A.</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Sociedade Corretora de TVM</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>São Paulo</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>Banco/CTVM</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>OUVIDORIA@CGDSECURITIES.COM.BR</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>11 30739300</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" s="3" t="inlineStr"/>
-      <c r="P51" s="3" t="inlineStr"/>
-      <c r="Q51" s="3" t="inlineStr"/>
-      <c r="R51" s="3" t="inlineStr"/>
-      <c r="S51" s="3" t="inlineStr"/>
-      <c r="T51" s="3" t="inlineStr"/>
-      <c r="U51" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:U51"/>
+  <autoFilter ref="A1:U45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>